<commit_message>
fix(dashboard): repair Expenses/Net Savings cell refs, rebuild clean buyer ZIP, update brand to Nivora
- Dashboard B40(=B4->=B5) Expenses now points to Total Expenses cell
- Dashboard B41(=B5->=B7) Net Savings now points to Net Savings cell
- Applied fix to both delivery/budget-planner-expense-tracker.xlsx and source artifact v1.2
- Rebuilt delivery ZIP with only 3 buyer files (xlsx, pdf, copy-link.txt)
- Updated google-sheets-copy-link.txt with final Nivora-branded content
- Added FINAL_ZIP_QA.md
- Updated PRODUCT_CATALOG.csv status to Ready to Publish
- Updated all context/continuation files with Nivora brand
- Created PRODUCT_FACTORY_CONTINUATION_CONTEXT.md
</commit_message>
<xml_diff>
--- a/01-product-factory/02-products/budget-planner-expense-tracker/artifacts/budget-planner-expense-tracker-v1.2.xlsx
+++ b/01-product-factory/02-products/budget-planner-expense-tracker/artifacts/budget-planner-expense-tracker-v1.2.xlsx
@@ -3261,7 +3261,7 @@
         </is>
       </c>
       <c r="B40" s="38">
-        <f>B4</f>
+        <f>B5</f>
         <v/>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
         </is>
       </c>
       <c r="B41" s="38">
-        <f>B5</f>
+        <f>B7</f>
         <v/>
       </c>
     </row>

</xml_diff>